<commit_message>
D6 for Table 1 updated
</commit_message>
<xml_diff>
--- a/i_test/test_D6_Tabella_1_fasciaeta_2025/g_output/D6_Table_1_40-64.xlsx
+++ b/i_test/test_D6_Tabella_1_fasciaeta_2025/g_output/D6_Table_1_40-64.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -375,6 +375,11 @@
           <t>SE</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Tutte</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -397,6 +402,11 @@
           <t>SE</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Tutte</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -406,17 +416,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>562</t>
+          <t>581</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>557</t>
+          <t>555</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>550</t>
+          <t>533</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1669</t>
         </is>
       </c>
     </row>
@@ -428,17 +443,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>289 (51,4%)</t>
+          <t>296 (50,9%)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>278 (49,9%)</t>
+          <t>274 (49,4%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>292 (53,1%)</t>
+          <t>289 (54,2%)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>859 (51,5%)</t>
         </is>
       </c>
     </row>
@@ -450,17 +470,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>50 (8,9%)</t>
+          <t>42 (7,2%)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>51 (9,2%)</t>
+          <t>40 (7,2%)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>55 (10,0%)</t>
+          <t>46 (8,6%)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>128 (7,7%)</t>
         </is>
       </c>
     </row>
@@ -474,110 +499,135 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>A10BD09</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>183 (32,6%)</t>
+          <t>A10BH 226 (0,4%)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>178 (32,0%)</t>
+          <t>A10BD07 219 (0,4%)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>169 (30,7%)</t>
+          <t>A10BD09 202 (0,4%)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>A10BD07 607 (0,4%)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>A10BK</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>198 (35,2%)</t>
+          <t>A10BD07 218 (0,4%)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>161 (28,9%)</t>
+          <t>A10AE56 212 (0,4%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>158 (28,7%)</t>
+          <t>A10AE54 200 (0,4%)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>A10BD10 603 (0,4%)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>A10BD24</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>178 (31,7%)</t>
+          <t>A10BD24 214 (0,4%)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>176 (31,6%)</t>
+          <t>A10AE54 209 (0,4%)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>160 (29,1%)</t>
+          <t>A10BD10 198 (0,4%)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>A10BD09 597 (0,4%)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>A10BJ</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>170 (30,2%)</t>
+          <t>A10BD10 212 (0,4%)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>170 (30,5%)</t>
+          <t>A10BD20 204 (0,4%)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>157 (28,5%)</t>
+          <t>A10BD13 195 (0,4%)</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>A10AE54 592 (0,4%)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>A10BH</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>169 (30,1%)</t>
+          <t>A10AE56 208 (0,4%)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>173 (31,1%)</t>
+          <t>A10BJ 203 (0,4%)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>154 (28,0%)</t>
+          <t>A10BX16 194 (0,4%)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>A10BH 590 (0,4%)</t>
         </is>
       </c>
     </row>
@@ -596,17 +646,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>258 (45,9%)</t>
+          <t>3 (0,5%)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>254 (45,6%)</t>
+          <t>5 (0,9%)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>283 (51,5%)</t>
+          <t>5 (0,9%)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>13 (0,8%)</t>
         </is>
       </c>
     </row>
@@ -625,17 +680,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>400 (71,2%)</t>
+          <t>367 (63,2%)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>376 (67,5%)</t>
+          <t>357 (64,3%)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>381 (69,3%)</t>
+          <t>339 (63,6%)</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>1.063 (63,7%)</t>
         </is>
       </c>
     </row>
@@ -647,17 +707,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>394 (70,1%)</t>
+          <t>61 (10,5%)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>358 (64,3%)</t>
+          <t>45 (8,1%)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>361 (65,6%)</t>
+          <t>63 (11,8%)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>169 (10,1%)</t>
         </is>
       </c>
     </row>
@@ -669,17 +734,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>132 (23,5%)</t>
+          <t>370 (63,7%)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>119 (21,4%)</t>
+          <t>353 (63,6%)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>125 (22,7%)</t>
+          <t>352 (66,0%)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>1.075 (64,4%)</t>
         </is>
       </c>
     </row>
@@ -691,17 +761,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>321 (57,1%)</t>
+          <t>268 (46,1%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>308 (55,3%)</t>
+          <t>233 (42,0%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>321 (58,4%)</t>
+          <t>226 (42,4%)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>727 (43,6%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
dataset including description of drugs simulated and D5 for Table 1 modified having description instead of ATC codes
</commit_message>
<xml_diff>
--- a/i_test/test_D6_Tabella_1_fasciaeta_2025/g_output/D6_Table_1_40-64.xlsx
+++ b/i_test/test_D6_Tabella_1_fasciaeta_2025/g_output/D6_Table_1_40-64.xlsx
@@ -504,22 +504,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>A10BH 226 (0,4%)</t>
+          <t>NA 226 (38,9%)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>A10BD07 219 (0,4%)</t>
+          <t>kk 219 (39,5%)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>A10BD09 202 (0,4%)</t>
+          <t>mm 202 (37,9%)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>A10BD07 607 (0,4%)</t>
+          <t>kk 607 (36,4%)</t>
         </is>
       </c>
     </row>
@@ -531,22 +531,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>A10BD07 218 (0,4%)</t>
+          <t>kk 218 (37,5%)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>A10AE56 212 (0,4%)</t>
+          <t>nn 212 (38,2%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>A10AE54 200 (0,4%)</t>
+          <t>oo 200 (37,5%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>A10BD10 603 (0,4%)</t>
+          <t>jj 603 (36,1%)</t>
         </is>
       </c>
     </row>
@@ -558,22 +558,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>A10BD24 214 (0,4%)</t>
+          <t>ee 214 (36,8%)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>A10AE54 209 (0,4%)</t>
+          <t>oo 209 (37,7%)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>A10BD10 198 (0,4%)</t>
+          <t>jj 198 (37,1%)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>A10BD09 597 (0,4%)</t>
+          <t>mm 597 (35,8%)</t>
         </is>
       </c>
     </row>
@@ -585,22 +585,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A10BD10 212 (0,4%)</t>
+          <t>jj 212 (36,5%)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>A10BD20 204 (0,4%)</t>
+          <t>rr 204 (36,8%)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>A10BD13 195 (0,4%)</t>
+          <t>hh 195 (36,6%)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>A10AE54 592 (0,4%)</t>
+          <t>oo 592 (35,5%)</t>
         </is>
       </c>
     </row>
@@ -612,22 +612,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A10AE56 208 (0,4%)</t>
+          <t>nn 208 (35,8%)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>A10BJ 203 (0,4%)</t>
+          <t>NA 203 (36,6%)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>A10BX16 194 (0,4%)</t>
+          <t>cc 194 (36,4%)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>A10BH 590 (0,4%)</t>
+          <t>NA 590 (35,4%)</t>
         </is>
       </c>
     </row>

</xml_diff>